<commit_message>
Retrieval accuracy improvements: bigger embedding model, hybrid search, prompt fixes. Final v1, deployment evaluated and deliberately not pursued.
</commit_message>
<xml_diff>
--- a/eval/qa_test_set.xlsx
+++ b/eval/qa_test_set.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KHUSHI\Desktop\My projects\Company Report Assistant\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\KHUSHI\Desktop\My projects\Company Report Assistant\eval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F2BFA5-A000-41DA-89E6-A66ED6142469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE61867-8104-426E-B8B8-8B1BF5FDA63A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="107">
   <si>
     <t>Company Report Assistant — Manual Evaluation Set</t>
   </si>
@@ -275,6 +275,93 @@
 Setting appropriate risk limits and controls.
 Monitoring such risks and compliance with the same.
 These risk management processes are reviewed regularly to reflect changes in market conditions and the Company's activities.</t>
+  </si>
+  <si>
+    <t>Updated Model Answer (from app)</t>
+  </si>
+  <si>
+    <t>HDFC Bank's capital adequacy ratio as of March 31, 2026, is 19.71%, and the Gross Non Performing Asset (GNPA) ratio is 2.44%.</t>
+  </si>
+  <si>
+    <t>According to the context provided, I was unable to find the specific amount spent on CSR initiatives in the report. However, I can tell you that the Bank completed 156 mandatory Impact Assessment studies and covered 498 border villages through rural development initiatives.</t>
+  </si>
+  <si>
+    <t>According to the report, HDFC Bank is using AI to handle customer queries and requests by leveraging Gen AI to "resolve Zero fraud onboarding and servicing" and to "improve customer queries and resolve customer queries and improve customers while ensuring privacy-resolution TAT. by-design."</t>
+  </si>
+  <si>
+    <t>According to the provided context, HDFC Bank's digital banking initiatives are anchored on five principles:
+FRICTIONLESS DIGITAL OMNICHANNEL CONSISTENCY CUSTOMER JOURNEYS EMPOWERMENT
+AI POWERED SAFE, SECURE, PERSONALISATION AND TRUSTWORTHY DIGITAL SERVICE BANKING
+Additionally, the bank is working on digital solutions to enhance productivity, widen and deepen wallet share from corporates, and create an ecosystem for seamless banking.</t>
+  </si>
+  <si>
+    <t>According to Page 112 of the report, HDFC Bank's approach to managing emerging risks is to operate in a dynamic environment where it maintains strong oversight, and uses secure and scalable platforms. It also acknowledges that human judgement remains central to decision-making, especially where customer impact is involved. The Bank remains vigilant to emerging risks, continuously assesses them through structured risk processes, and uses AI in a way that enhances efficiency while maintaining trust and control.</t>
+  </si>
+  <si>
+    <t>The context does not explicitly mention the specific macroeconomic developments highlighted by HDFC Bank's leadership for FY 2025-26. However, it does mention the Bank's focus on "accelerating credit and trade workflows, responsible innovation, strengthening transparency in decisioning, and reducing manual effort across teams" as part of its transformation initiatives.</t>
+  </si>
+  <si>
+    <t>According to the report, TCS's revenue growth in FY 2026 was 4.6% on a reported basis, and in constant currency, it was a decline of 2.4%. On the other hand, the operating margin in FY 2026 was 25.0%.</t>
+  </si>
+  <si>
+    <t>TCS believes that every employee should have access to market relevant learning opportunities. They value their people and have a culture that helps create a strong sense of belonging. They have a focused investments in building a future-ready workforce and nurturing leaders from within, which has developed a robust management pipeline.</t>
+  </si>
+  <si>
+    <t>TCS announced partnerships around AI with the following companies:
+OpenAI
+AMD
+ABB
+Honeywell
+Google Cloud</t>
+  </si>
+  <si>
+    <t>According to the context provided, HUL describes its impact on rural India as part of its broader commitment to sustainable living and responsible business growth. In the CSR section, it mentions that its CSR initiatives in aspirational districts have delivered measurable improvements in livelihoods, water and waste management, and other critical development areas, contributing to better quality of life and sustainable regional development. This indicates that HUL views its impact in rural India as positive and focused on improving the lives of vulnerable groups such as women, children, and the elderly.</t>
+  </si>
+  <si>
+    <t>According to the context, HUL mentioned that they have strong momentum in their Coffee and Lifestyle Nutrition segments, which are "premium, purpose-led and culturally relevant", indicating a positive performance of these new brands.</t>
+  </si>
+  <si>
+    <t>Reliance described Reliance Retail as the "largest integrated omni-channel retailer in India" and stated that it is "the largest player in distribution" and has a "large and growing customer franchise supported by consumer preferences".</t>
+  </si>
+  <si>
+    <t>Reliance plans to establish and enable 100 GW of renewable energy capacity by 2030, with a focus on developing a 6 GWp solar power project by 2035.</t>
+  </si>
+  <si>
+    <t>According to the report, Jio's digital business performed exceptionally well financially in FY 2025-26, with Revenue and EBITDA growth of 14.3% and 17.8% year-over-year, respectively.</t>
+  </si>
+  <si>
+    <t>According to Page 37 of the report, the US business contributed 29% of consolidated revenues in FY26. The revenue generated by the US business was ₹ 168.2 Billion, which is an increase of 3.6% from the previous year.</t>
+  </si>
+  <si>
+    <t>According to the context provided, Sun Pharma has a risk management assessment and policies and processes in place to identify and analyze financial risks, set appropriate risk limits and controls, and monitor such risks and compliance with the same. The risk management policy includes a framework for identifying internal and external risks related to cybersecurity or information hazards. The synopsis of the policy can be accessed at the provided web-link.</t>
+  </si>
+  <si>
+    <t>I couldn't find that information in the report.</t>
+  </si>
+  <si>
+    <t>Updated Model Answer (from app) 2.0</t>
+  </si>
+  <si>
+    <t>According to the report, HDFC Bank spent 1,316.18 crore on CSR initiatives. However, I couldn't find information on the exact number of villages where HDFC Bank has a presence. The report does provide details on the CSR projects, which include various initiatives such as rural development, skill training, and education, but it does not specify the number of villages involved.</t>
+  </si>
+  <si>
+    <t>HDFC Bank is using AI to handle customer queries and requests by powering advanced customer analytics that identify the right customer, channel, product offering, and personalize communication, lead prioritization, and engagement. This has enabled employees to handle customer queries and service requests more efficiently, delivering faster and more consistent responses. AI-powered behavioral insights, including digital engagement and drop-solutions, have also been used to simplify and streamline operations, significantly reducing manual effort and response times.</t>
+  </si>
+  <si>
+    <t>TCS views its workforce and talent development as crucial to its success. According to the report, the company aims to create a future-ready workforce that is equipped with the skills needed to drive its transformation into an AI-first enterprise. To achieve this, TCS invests in building a heterogeneous workforce and providing market-relevant learning opportunities to all its employees. The company also places a strong emphasis on nurturing leaders from within, with a robust management pipeline that supports seamless succession into senior leadership roles. Additionally, TCS has implemented various initiatives, such as its "Best in Class Talent Management" program, to attract and retain top talent, including specialized hiring, external certifications, and consulting expertise.</t>
+  </si>
+  <si>
+    <t>TCS announced two new partnerships around AI: one with Google Cloud, which involves adopting its next-generation agentic AI platform, Gemini Enterprise. This partnership aims to empower TCS' workforce to build agentic AI solutions to redefine Human + AI workflows.
+Additionally, TCS announced a collaboration with AMD, which includes co-developing a rack-scale AI infrastructure design based on the AMD 'Helios' platform. This partnership also aims to enhance market access and provide an AI-ready data center blueprint with capacities of up to 200 MW.</t>
+  </si>
+  <si>
+    <t>Reliance plans to establish and enable 100 GW of solar power capacity by 2030, with an initial target of 6 GWp by 2035, and a planned capacity of 20 GWp by 2030, with the goal of producing 40 GWh of annual capacity.</t>
+  </si>
+  <si>
+    <t>Sun Pharma has launched two notable drugs in the US market: UNLOXCYT, a treatment for adults with metastatic cutaneous squamous cell carcinoma or locally advanced cutaneous squamous cell carcinoma, and LEQSELVI, a treatment for severe alopecia areata.</t>
+  </si>
+  <si>
+    <t>According to the context, HUL announced the development of a state-of-the-art digital manufacturing center for Bars, which includes a pilot plant that replicates global manufacturing processes. This will enable scientists to prototype and refine new formats more efficiently, thereby enhancing the company's manufacturing capabilities.</t>
   </si>
 </sst>
 </file>
@@ -366,15 +453,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -392,6 +470,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -695,54 +782,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
     <col min="3" max="3" width="44.88671875" customWidth="1"/>
     <col min="4" max="4" width="45.88671875" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="34" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" customWidth="1"/>
-    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="6" max="7" width="34" customWidth="1"/>
+    <col min="8" max="8" width="38.5546875" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:10" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -762,412 +856,504 @@
         <v>7</v>
       </c>
       <c r="G4" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
+    <row r="5" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
         <v>1</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="G5" s="9"/>
-      <c r="H5" s="8"/>
-    </row>
-    <row r="6" spans="1:8" ht="72" x14ac:dyDescent="0.3">
-      <c r="A6" s="6">
+      <c r="G5" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="5"/>
+    </row>
+    <row r="6" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
         <v>2</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="9"/>
-      <c r="H6" s="8"/>
-    </row>
-    <row r="7" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="6">
+      <c r="G6" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I6" s="6"/>
+      <c r="J6" s="5"/>
+    </row>
+    <row r="7" spans="1:10" ht="222.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="G7" s="9"/>
-      <c r="H7" s="8"/>
-    </row>
-    <row r="8" spans="1:8" ht="144" x14ac:dyDescent="0.3">
-      <c r="A8" s="6">
+      <c r="G7" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I7" s="6"/>
+      <c r="J7" s="5"/>
+    </row>
+    <row r="8" spans="1:10" ht="250.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="G8" s="9"/>
-      <c r="H8" s="8"/>
-    </row>
-    <row r="9" spans="1:8" ht="144" x14ac:dyDescent="0.3">
-      <c r="A9" s="6">
+      <c r="G8" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H8" s="5"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="5"/>
+    </row>
+    <row r="9" spans="1:10" ht="232.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>5</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G9" s="9"/>
-      <c r="H9" s="8"/>
-    </row>
-    <row r="10" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="6">
+      <c r="G9" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="H9" s="5"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="5"/>
+    </row>
+    <row r="10" spans="1:10" ht="181.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>6</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="G10" s="9"/>
-      <c r="H10" s="8"/>
-    </row>
-    <row r="11" spans="1:8" ht="72" x14ac:dyDescent="0.3">
-      <c r="A11" s="6">
+      <c r="G10" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H10" s="5"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="5"/>
+    </row>
+    <row r="11" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>7</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G11" s="9"/>
-      <c r="H11" s="8"/>
-    </row>
-    <row r="12" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="6">
+      <c r="G11" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="H11" s="5"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="5"/>
+    </row>
+    <row r="12" spans="1:10" ht="297" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>8</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="G12" s="9"/>
-      <c r="H12" s="8"/>
-    </row>
-    <row r="13" spans="1:8" ht="216" x14ac:dyDescent="0.3">
-      <c r="A13" s="6">
+      <c r="G12" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="I12" s="6"/>
+      <c r="J12" s="5"/>
+    </row>
+    <row r="13" spans="1:10" ht="257.39999999999998" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>9</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G13" s="9"/>
-      <c r="H13" s="8"/>
-    </row>
-    <row r="14" spans="1:8" ht="144" x14ac:dyDescent="0.3">
-      <c r="A14" s="6">
+      <c r="G13" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="I13" s="6"/>
+      <c r="J13" s="5"/>
+    </row>
+    <row r="14" spans="1:10" ht="270.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <v>10</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G14" s="9"/>
-      <c r="H14" s="8"/>
-    </row>
-    <row r="15" spans="1:8" ht="52.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="6">
+      <c r="G14" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="H14" s="5"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="5"/>
+    </row>
+    <row r="15" spans="1:10" ht="136.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <v>11</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G15" s="9"/>
-      <c r="H15" s="8"/>
-    </row>
-    <row r="16" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="6">
+      <c r="G15" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="I15" s="6"/>
+      <c r="J15" s="5"/>
+    </row>
+    <row r="16" spans="1:10" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <v>12</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="G16" s="9"/>
-      <c r="H16" s="8"/>
-    </row>
-    <row r="17" spans="1:8" ht="273.60000000000002" x14ac:dyDescent="0.3">
-      <c r="A17" s="6">
+      <c r="G16" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="5"/>
+    </row>
+    <row r="17" spans="1:10" ht="307.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>13</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G17" s="9"/>
-      <c r="H17" s="8"/>
-    </row>
-    <row r="18" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="6">
+      <c r="G17" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="H17" s="5"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="5"/>
+    </row>
+    <row r="18" spans="1:10" ht="121.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
         <v>14</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G18" s="9"/>
-      <c r="H18" s="8"/>
-    </row>
-    <row r="19" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="6">
+      <c r="G18" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="I18" s="6"/>
+      <c r="J18" s="5"/>
+    </row>
+    <row r="19" spans="1:10" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
         <v>15</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="9"/>
-      <c r="H19" s="8"/>
-    </row>
-    <row r="20" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="6">
+      <c r="G19" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="H19" s="5"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="5"/>
+    </row>
+    <row r="20" spans="1:10" ht="129" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
         <v>16</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="G20" s="9"/>
-      <c r="H20" s="8"/>
-    </row>
-    <row r="21" spans="1:8" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="6">
+      <c r="G20" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H20" s="5"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" spans="1:10" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
         <v>17</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G21" s="9"/>
-      <c r="H21" s="8"/>
-    </row>
-    <row r="22" spans="1:8" ht="230.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="6">
+      <c r="G21" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I21" s="6"/>
+      <c r="J21" s="5"/>
+    </row>
+    <row r="22" spans="1:10" ht="243" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
         <v>18</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G22" s="9"/>
-      <c r="H22" s="8"/>
+      <c r="G22" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H22" s="5"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>